<commit_message>
update few shot exp
</commit_message>
<xml_diff>
--- a/data/describe/few_shot/cluster/messages_foot.xlsx
+++ b/data/describe/few_shot/cluster/messages_foot.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\input_cluster\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amaca253\Documents\datomatisation\datomatisation-dev\data\describe\few_shot\cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B82F796-04EE-4D19-A6FE-ED7F5AEE4BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A7F34B-2165-4E05-A1B6-002E398E4B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34950" yWindow="570" windowWidth="34065" windowHeight="17070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51855" yWindow="2955" windowWidth="20190" windowHeight="17070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>User</t>
   </si>
@@ -45,23 +45,6 @@
     <t>A creative maestro is a player who constantly delivers dangerous passes in the attacking third, always finding space to receive the ball in crucial attacking positions, and threading ingenious smart passes while making crucial key passes. These players are also very strong in winning ground duels, demonstrating their ability to both create opportunities and fight for possession.</t>
   </si>
   <si>
-    <t xml:space="preserve">Now your task is to provide a description of a cluster.
-You will receive information about the cluster based on the latent factors that best describe it.
-For each cluster, write a concise summary based on the available information.
-The first sentence should give an overview of the cluster. 
-The second sentence should describe the cluster’s specific strengths based on the available information.
-The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
-I will provided you with the cluster description and you will return the summary. </t>
-  </si>
-  <si>
-    <t>Understood. Please provide the cluster descriptions.</t>
-  </si>
-  <si>
-    <t>This cluster describes players who are exceptionally strong goal producers, while being average in their aerial abilities.
-Their primary strength lies in their prolific goal-scoring capability and consistent ability to generate high-quality scoring chances, regardless of playing time.
-A potential weakness is their average performance in aerial duels, meaning they are not particularly dominant when the ball is contested high in the air.</t>
-  </si>
-  <si>
     <t>What does it mean when a football player is described as goal-shy?</t>
   </si>
   <si>
@@ -72,29 +55,6 @@
   </si>
   <si>
     <t>A prolific scorer is a player who truly knows how to find the back of the net, consistently delivering a high volume of goals per 90 minutes, even when we strip away penalties. These players also tend to enjoy significant time on the field, which gives them ample opportunity to showcase their exceptional scoring ability.</t>
-  </si>
-  <si>
-    <t>This cluster describes players who are prolific and consistent goal-scorers, although they exhibit a slight weakness in winning aerial duels.
-Their primary strength lies in their exceptional goal-scoring ability, consistently finding the back of the net and making every minute on the pitch count for scoring opportunities.
-However, they exhibit a slight weakness in aerial duels, meaning they are less likely to win contested balls in the air and may not be a significant threat from crosses or set pieces.</t>
-  </si>
-  <si>
-    <t>This cluster describes players who are generally not dominant in aerial duels and exhibit an average tendency to be goal-shy.
-Based on the provided factors, this cluster does not exhibit specific strengths in goal contribution or aerial ability.
-Their clear weaknesses include a marked inability to win aerial duels and a consistent lack of prolific scoring, meaning they are less impactful in situations requiring heading or regular goal production.</t>
-  </si>
-  <si>
-    <t>This cluster describes players who are exceptionally skilled at orchestrating attacks and creating chances, while maintaining a reliable, albeit not extraordinary, goal-scoring presence.
-Their paramount strength lies in their extraordinary capacity as a creative maestro, consistently dazzling with incisive passes, unlocking defenses, and winning crucial ground duels to drive their team's attack.
-However, while their goal-scoring is consistent, it remains at a normal level, indicating they are not exceptionally prolific in front of goal, especially when compared to their elite playmaking abilities.</t>
-  </si>
-  <si>
-    <t>This cluster represents players who are strong contributors to their team's attack, blending solid creative playmaking with a notable inclination to find the back of the net.
-Their specific strengths lie in their above-average ability to deliver dangerous passes, find crucial attacking space, and win ground duels, alongside a clear tendency to score goals and gain significant playing time.
-While highly effective, their creativity, though strong, doesn't reach the absolute pinnacle of a "maestro," suggesting they are consistently good but perhaps not always the most ingenious in every attacking phase.</t>
-  </si>
-  <si>
-    <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical football player in that cluster: ```Members of this cluster can be described as:  slightly low on good in air,  very low on goal-shy´´´</t>
   </si>
   <si>
     <t>Here is the cluster description based on the factor scores at the cluster center, representing a typical football player in that cluster:```Members of this cluster can be described as:  normal on good in air,  quite high on prolific scorer´´´</t>
@@ -115,6 +75,44 @@
 The second sentence should describe the cluster’s specific strengths based on the available information.
 The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
 Now do the same thing with the following: ```Members of this cluster can be described as:  slightly high on creative maestro,  slightly low on goal-shy´´´</t>
+  </si>
+  <si>
+    <t>Thats really good. You truly understand the factors and names. 
+Now your task is to provide a description of a cluster.
+Please use the statistical description enclosed with ``` ´´´ . It provides information about the cluster based on the latent factors that most accurately describe it.
+Now your task is to provide a description of a cluster.
+You will receive information about the cluster based on the latent factors that best describe it.
+For each cluster, write a concise summary based on the available information.
+The first sentence should give an overview of the cluster. 
+The second sentence should describe the cluster’s specific strengths based on the available information.
+The third sentence should highlight areas where the cluster has specific weaknesses based on the available information.
+I will provided you with the cluster description and you will return the summary. 
+Here is the cluster description based on the factor scores at the cluster center, representing a typical football player in that cluster: ```Members of this cluster can be described as:  slightly low on good in air,  very low on goal-shy´´´</t>
+  </si>
+  <si>
+    <t>This cluster describes players who are prolific and consistent goal-scorers, although they exhibit a slight weakness in winning aerial duels.
+Their primary strength lies in their exceptional goal-scoring ability, consistently finding the back of the net and making every minute on the pitch count for scoring opportunities.
+However, they exhibit a slight weakness in aerial duels, meaning they are less likely to win contested balls in the air and may not be a significant threat from crosses or set pieces.</t>
+  </si>
+  <si>
+    <t>This cluster describes players who are exceptionally strong goal producers, while being average in their aerial abilities.
+Their primary strength lies in their prolific goal-scoring capability and consistent ability to generate high-quality scoring chances, regardless of playing time.
+A potential weakness is their average performance in aerial duels, meaning they are not particularly dominant when the ball is contested high in the air.</t>
+  </si>
+  <si>
+    <t>This cluster describes players who are generally not dominant in aerial duels and exhibit an average tendency to be goal-shy.
+Based on the provided factors, this cluster does not exhibit specific strengths in goal contribution or aerial ability.
+Their clear weaknesses include a marked inability to win aerial duels and a consistent lack of prolific scoring, meaning they are less impactful in situations requiring heading or regular goal production.</t>
+  </si>
+  <si>
+    <t>This cluster describes players who are exceptionally skilled at orchestrating attacks and creating chances, while maintaining a reliable, albeit not extraordinary, goal-scoring presence.
+Their paramount strength lies in their extraordinary capacity as a creative maestro, consistently dazzling with incisive passes, unlocking defenses, and winning crucial ground duels to drive their team's attack.
+However, while their goal-scoring is consistent, it remains at a normal level, indicating they are not exceptionally prolific in front of goal, especially when compared to their elite playmaking abilities.</t>
+  </si>
+  <si>
+    <t>This cluster represents players who are strong contributors to their team's attack, blending solid creative playmaking with a notable inclination to find the back of the net.
+Their specific strengths lie in their above-average ability to deliver dangerous passes, find crucial attacking space, and win ground duels, alongside a clear tendency to score goals and gain significant playing time.
+While highly effective, their creativity, though strong, doesn't reach the absolute pinnacle of a "maestro," suggesting they are consistently good but perhaps not always the most ingenious in every attacking phase.</t>
   </si>
 </sst>
 </file>
@@ -483,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="94.26953125" style="2" customWidth="1"/>
@@ -516,66 +514,58 @@
     </row>
     <row r="4" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="87" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="116" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="116" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="B7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="116" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>